<commit_message>
Casi termine descriptivo AgbA (falta probar que es paseo aleatorio con los TH)
</commit_message>
<xml_diff>
--- a/Informe/Tablas/tabla_covs.xlsx
+++ b/Informe/Tablas/tabla_covs.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="49">
   <si>
     <t>Variable</t>
   </si>
@@ -178,6 +178,12 @@
   </si>
   <si>
     <t>Fecha de la observación</t>
+  </si>
+  <si>
+    <t>Cerdo</t>
+  </si>
+  <si>
+    <t>Precio de la carne porcina</t>
   </si>
 </sst>
 </file>
@@ -519,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.7265625" customWidth="1"/>
@@ -682,8 +688,11 @@
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>15</v>
+      <c r="A15" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" t="s">
+        <v>48</v>
       </c>
       <c r="C15" t="s">
         <v>23</v>
@@ -691,10 +700,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>16</v>
-      </c>
-      <c r="B16" t="s">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="C16" t="s">
         <v>23</v>
@@ -702,10 +708,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C17" t="s">
         <v>23</v>
@@ -713,29 +719,32 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="C18" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C19" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>20</v>
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>35</v>
       </c>
       <c r="C20" t="s">
         <v>23</v>
@@ -743,20 +752,28 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C21" t="s">
-        <v>42</v>
+        <v>23</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>22</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B23" t="s">
         <v>37</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C23" t="s">
         <v>36</v>
       </c>
     </row>

</xml_diff>